<commit_message>
Add menu item photos and Uber Eats ordering
</commit_message>
<xml_diff>
--- a/outputs/menu/menu.xlsx
+++ b/outputs/menu/menu.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R36fcb22d2362470f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items" sheetId="2" r:id="R211b8311a34d44da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories" sheetId="3" r:id="Rf592561c0b324341"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="option_groups" sheetId="4" r:id="R22b2d482d42a4d30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="options" sheetId="5" r:id="R67c1f55ea86f45be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="specials" sheetId="6" r:id="Rea060350f0f24488"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hours" sheetId="7" r:id="Rd6d8be6982734eb0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="site_settings" sheetId="8" r:id="R777f556cb5964619"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R1b3bc90ba0d8447d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items" sheetId="2" r:id="Reefa5ba854394f94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories" sheetId="3" r:id="Rb29171e6e1764327"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="option_groups" sheetId="4" r:id="R7f616509418d4c81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="options" sheetId="5" r:id="Ra22121c5f8bb4ec1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="specials" sheetId="6" r:id="Rc09021ada29240f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hours" sheetId="7" r:id="R4f9c26f23e704d09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="site_settings" sheetId="8" r:id="R88c8d79a1dad4ed9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -221,7 +221,7 @@
     <x:tableColumn id="6" name="cta_primary_text_fi"/>
     <x:tableColumn id="7" name="cta_primary_link"/>
     <x:tableColumn id="8" name="external_order_wolt_url"/>
-    <x:tableColumn id="9" name="external_order_foodora_url"/>
+    <x:tableColumn id="9" name="external_order_uber_eats_url"/>
     <x:tableColumn id="10" name="phone"/>
     <x:tableColumn id="11" name="email"/>
     <x:tableColumn id="12" name="address_line1"/>
@@ -506,7 +506,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R811a953eca4340c9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca35dd4503c84583"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -649,7 +649,9 @@
       <x:c r="S2" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T2" s="1" t="str"/>
+      <x:c r="T2" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01253.jpg</x:v>
+      </x:c>
       <x:c r="U2" s="1" t="str"/>
       <x:c r="V2" s="1" t="str"/>
     </x:row>
@@ -695,7 +697,9 @@
       <x:c r="S3" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T3" s="1" t="str"/>
+      <x:c r="T3" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01263.jpg</x:v>
+      </x:c>
       <x:c r="U3" s="1" t="str"/>
       <x:c r="V3" s="1" t="str"/>
     </x:row>
@@ -741,7 +745,9 @@
       <x:c r="S4" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T4" s="1" t="str"/>
+      <x:c r="T4" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01266.jpg</x:v>
+      </x:c>
       <x:c r="U4" s="1" t="str"/>
       <x:c r="V4" s="1" t="str"/>
     </x:row>
@@ -787,7 +793,9 @@
       <x:c r="S5" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T5" s="1" t="str"/>
+      <x:c r="T5" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01283.jpg</x:v>
+      </x:c>
       <x:c r="U5" s="1" t="str"/>
       <x:c r="V5" s="1" t="str"/>
     </x:row>
@@ -833,7 +841,9 @@
       <x:c r="S6" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T6" s="1" t="str"/>
+      <x:c r="T6" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01287.jpg</x:v>
+      </x:c>
       <x:c r="U6" s="1" t="str"/>
       <x:c r="V6" s="1" t="str"/>
     </x:row>
@@ -879,7 +889,9 @@
       <x:c r="S7" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T7" s="1" t="str"/>
+      <x:c r="T7" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01291.jpg</x:v>
+      </x:c>
       <x:c r="U7" s="1" t="str"/>
       <x:c r="V7" s="1" t="str"/>
     </x:row>
@@ -925,7 +937,9 @@
       <x:c r="S8" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T8" s="1" t="str"/>
+      <x:c r="T8" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01297.jpg</x:v>
+      </x:c>
       <x:c r="U8" s="1" t="str"/>
       <x:c r="V8" s="1" t="str"/>
     </x:row>
@@ -971,7 +985,9 @@
       <x:c r="S9" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T9" s="1" t="str"/>
+      <x:c r="T9" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01301.jpg</x:v>
+      </x:c>
       <x:c r="U9" s="1" t="str"/>
       <x:c r="V9" s="1" t="str"/>
     </x:row>
@@ -1017,7 +1033,9 @@
       <x:c r="S10" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T10" s="1" t="str"/>
+      <x:c r="T10" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01304.jpg</x:v>
+      </x:c>
       <x:c r="U10" s="1" t="str"/>
       <x:c r="V10" s="1" t="str"/>
     </x:row>
@@ -1063,7 +1081,9 @@
       <x:c r="S11" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T11" s="1" t="str"/>
+      <x:c r="T11" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01308.jpg</x:v>
+      </x:c>
       <x:c r="U11" s="1" t="str"/>
       <x:c r="V11" s="1" t="str"/>
     </x:row>
@@ -1107,7 +1127,9 @@
       <x:c r="S12" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T12" s="1" t="str"/>
+      <x:c r="T12" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01310.jpg</x:v>
+      </x:c>
       <x:c r="U12" s="1" t="str"/>
       <x:c r="V12" s="1" t="str"/>
     </x:row>
@@ -1153,7 +1175,9 @@
       <x:c r="S13" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T13" s="1" t="str"/>
+      <x:c r="T13" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01314.jpg</x:v>
+      </x:c>
       <x:c r="U13" s="1" t="str"/>
       <x:c r="V13" s="1" t="str"/>
     </x:row>
@@ -1199,7 +1223,9 @@
       <x:c r="S14" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T14" s="1" t="str"/>
+      <x:c r="T14" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01318.jpg</x:v>
+      </x:c>
       <x:c r="U14" s="1" t="str"/>
       <x:c r="V14" s="1" t="str"/>
     </x:row>
@@ -1245,7 +1271,9 @@
       <x:c r="S15" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T15" s="1" t="str"/>
+      <x:c r="T15" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01340.jpg</x:v>
+      </x:c>
       <x:c r="U15" s="1" t="str"/>
       <x:c r="V15" s="1" t="str"/>
     </x:row>
@@ -1291,7 +1319,9 @@
       <x:c r="S16" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T16" s="1" t="str"/>
+      <x:c r="T16" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01348.jpg</x:v>
+      </x:c>
       <x:c r="U16" s="1" t="str"/>
       <x:c r="V16" s="1" t="str"/>
     </x:row>
@@ -1337,7 +1367,9 @@
       <x:c r="S17" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T17" s="1" t="str"/>
+      <x:c r="T17" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01353.jpg</x:v>
+      </x:c>
       <x:c r="U17" s="1" t="str"/>
       <x:c r="V17" s="1" t="str"/>
     </x:row>
@@ -1383,7 +1415,9 @@
       <x:c r="S18" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T18" s="1" t="str"/>
+      <x:c r="T18" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01355.jpg</x:v>
+      </x:c>
       <x:c r="U18" s="1" t="str"/>
       <x:c r="V18" s="1" t="str"/>
     </x:row>
@@ -1429,7 +1463,9 @@
       <x:c r="S19" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T19" s="1" t="str"/>
+      <x:c r="T19" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01360.jpg</x:v>
+      </x:c>
       <x:c r="U19" s="1" t="str"/>
       <x:c r="V19" s="1" t="str"/>
     </x:row>
@@ -1487,7 +1523,9 @@
       <x:c r="S20" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T20" s="1" t="str"/>
+      <x:c r="T20" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01371.jpg</x:v>
+      </x:c>
       <x:c r="U20" s="1" t="str"/>
       <x:c r="V20" s="1" t="str"/>
     </x:row>
@@ -1545,7 +1583,9 @@
       <x:c r="S21" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T21" s="1" t="str"/>
+      <x:c r="T21" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01374.jpg</x:v>
+      </x:c>
       <x:c r="U21" s="1" t="str"/>
       <x:c r="V21" s="1" t="str"/>
     </x:row>
@@ -1603,7 +1643,9 @@
       <x:c r="S22" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T22" s="1" t="str"/>
+      <x:c r="T22" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01380.jpg</x:v>
+      </x:c>
       <x:c r="U22" s="1" t="str"/>
       <x:c r="V22" s="1" t="str"/>
     </x:row>
@@ -1649,7 +1691,9 @@
       <x:c r="S23" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T23" s="1" t="str"/>
+      <x:c r="T23" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01386.jpg</x:v>
+      </x:c>
       <x:c r="U23" s="1" t="str"/>
       <x:c r="V23" s="1" t="str"/>
     </x:row>
@@ -1693,7 +1737,9 @@
       <x:c r="S24" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T24" s="1" t="str"/>
+      <x:c r="T24" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01387.jpg</x:v>
+      </x:c>
       <x:c r="U24" s="1" t="str"/>
       <x:c r="V24" s="1" t="str"/>
     </x:row>
@@ -1737,7 +1783,9 @@
       <x:c r="S25" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T25" s="1" t="str"/>
+      <x:c r="T25" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01389.jpg</x:v>
+      </x:c>
       <x:c r="U25" s="1" t="str"/>
       <x:c r="V25" s="1" t="str"/>
     </x:row>
@@ -1781,7 +1829,9 @@
       <x:c r="S26" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T26" s="1" t="str"/>
+      <x:c r="T26" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01392.jpg</x:v>
+      </x:c>
       <x:c r="U26" s="1" t="str"/>
       <x:c r="V26" s="1" t="str"/>
     </x:row>
@@ -1825,7 +1875,9 @@
       <x:c r="S27" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T27" s="1" t="str"/>
+      <x:c r="T27" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01394.jpg</x:v>
+      </x:c>
       <x:c r="U27" s="1" t="str"/>
       <x:c r="V27" s="1" t="str"/>
     </x:row>
@@ -1869,7 +1921,9 @@
       <x:c r="S28" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T28" s="1" t="str"/>
+      <x:c r="T28" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01395.jpg</x:v>
+      </x:c>
       <x:c r="U28" s="1" t="str"/>
       <x:c r="V28" s="1" t="str"/>
     </x:row>
@@ -1915,7 +1969,9 @@
       <x:c r="S29" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T29" s="1" t="str"/>
+      <x:c r="T29" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01401.jpg</x:v>
+      </x:c>
       <x:c r="U29" s="1" t="str"/>
       <x:c r="V29" s="1" t="str"/>
     </x:row>
@@ -1959,7 +2015,9 @@
       <x:c r="S30" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T30" s="1" t="str"/>
+      <x:c r="T30" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01402.jpg</x:v>
+      </x:c>
       <x:c r="U30" s="1" t="str"/>
       <x:c r="V30" s="1" t="str"/>
     </x:row>
@@ -2003,7 +2061,9 @@
       <x:c r="S31" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T31" s="1" t="str"/>
+      <x:c r="T31" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01417.jpg</x:v>
+      </x:c>
       <x:c r="U31" s="1" t="str"/>
       <x:c r="V31" s="1" t="str"/>
     </x:row>
@@ -2047,7 +2107,9 @@
       <x:c r="S32" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T32" s="1" t="str"/>
+      <x:c r="T32" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01419.jpg</x:v>
+      </x:c>
       <x:c r="U32" s="1" t="str"/>
       <x:c r="V32" s="1" t="str"/>
     </x:row>
@@ -2091,7 +2153,9 @@
       <x:c r="S33" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T33" s="1" t="str"/>
+      <x:c r="T33" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01423.jpg</x:v>
+      </x:c>
       <x:c r="U33" s="1" t="str"/>
       <x:c r="V33" s="1" t="str"/>
     </x:row>
@@ -2135,7 +2199,9 @@
       <x:c r="S34" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T34" s="1" t="str"/>
+      <x:c r="T34" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01425.jpg</x:v>
+      </x:c>
       <x:c r="U34" s="1" t="str"/>
       <x:c r="V34" s="1" t="str"/>
     </x:row>
@@ -2179,7 +2245,9 @@
       <x:c r="S35" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T35" s="1" t="str"/>
+      <x:c r="T35" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01430.jpg</x:v>
+      </x:c>
       <x:c r="U35" s="1" t="str"/>
       <x:c r="V35" s="1" t="str"/>
     </x:row>
@@ -2217,7 +2285,9 @@
       <x:c r="S36" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T36" s="1" t="str"/>
+      <x:c r="T36" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01433.jpg</x:v>
+      </x:c>
       <x:c r="U36" s="1" t="str"/>
       <x:c r="V36" s="1" t="str"/>
     </x:row>
@@ -2259,7 +2329,9 @@
       <x:c r="S37" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T37" s="1" t="str"/>
+      <x:c r="T37" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01438.jpg</x:v>
+      </x:c>
       <x:c r="U37" s="1" t="str"/>
       <x:c r="V37" s="1" t="str"/>
     </x:row>
@@ -2301,7 +2373,9 @@
       <x:c r="S38" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T38" s="1" t="str"/>
+      <x:c r="T38" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01447.jpg</x:v>
+      </x:c>
       <x:c r="U38" s="1" t="str"/>
       <x:c r="V38" s="1" t="str"/>
     </x:row>
@@ -2339,7 +2413,9 @@
       <x:c r="S39" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T39" s="1" t="str"/>
+      <x:c r="T39" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01456.jpg</x:v>
+      </x:c>
       <x:c r="U39" s="1" t="str"/>
       <x:c r="V39" s="1" t="str"/>
     </x:row>
@@ -2381,7 +2457,9 @@
       <x:c r="S40" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T40" s="1" t="str"/>
+      <x:c r="T40" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01462.jpg</x:v>
+      </x:c>
       <x:c r="U40" s="1" t="str"/>
       <x:c r="V40" s="1" t="str"/>
     </x:row>
@@ -2423,7 +2501,9 @@
       <x:c r="S41" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T41" s="1" t="str"/>
+      <x:c r="T41" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01466.jpg</x:v>
+      </x:c>
       <x:c r="U41" s="1" t="str"/>
       <x:c r="V41" s="1" t="str"/>
     </x:row>
@@ -2461,7 +2541,9 @@
       <x:c r="S42" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T42" s="1" t="str"/>
+      <x:c r="T42" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01468.jpg</x:v>
+      </x:c>
       <x:c r="U42" s="1" t="str"/>
       <x:c r="V42" s="1" t="str"/>
     </x:row>
@@ -2499,7 +2581,9 @@
       <x:c r="S43" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T43" s="1" t="str"/>
+      <x:c r="T43" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01469.jpg</x:v>
+      </x:c>
       <x:c r="U43" s="1" t="str"/>
       <x:c r="V43" s="1" t="str"/>
     </x:row>
@@ -2537,7 +2621,9 @@
       <x:c r="S44" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T44" s="1" t="str"/>
+      <x:c r="T44" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01473.jpg</x:v>
+      </x:c>
       <x:c r="U44" s="1" t="str"/>
       <x:c r="V44" s="1" t="str"/>
     </x:row>
@@ -2575,7 +2661,9 @@
       <x:c r="S45" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T45" s="1" t="str"/>
+      <x:c r="T45" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01481.jpg</x:v>
+      </x:c>
       <x:c r="U45" s="1" t="str"/>
       <x:c r="V45" s="1" t="str"/>
     </x:row>
@@ -2613,7 +2701,9 @@
       <x:c r="S46" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T46" s="1" t="str"/>
+      <x:c r="T46" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01488.jpg</x:v>
+      </x:c>
       <x:c r="U46" s="1" t="str"/>
       <x:c r="V46" s="1" t="str"/>
     </x:row>
@@ -2651,7 +2741,9 @@
       <x:c r="S47" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T47" s="1" t="str"/>
+      <x:c r="T47" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01492.jpg</x:v>
+      </x:c>
       <x:c r="U47" s="1" t="str"/>
       <x:c r="V47" s="1" t="str"/>
     </x:row>
@@ -2689,7 +2781,9 @@
       <x:c r="S48" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T48" s="1" t="str"/>
+      <x:c r="T48" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01501.jpg</x:v>
+      </x:c>
       <x:c r="U48" s="1" t="str"/>
       <x:c r="V48" s="1" t="str"/>
     </x:row>
@@ -2727,7 +2821,9 @@
       <x:c r="S49" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T49" s="1" t="str"/>
+      <x:c r="T49" s="1" t="str">
+        <x:v>assets/images/item-photos/TML01502.jpg</x:v>
+      </x:c>
       <x:c r="U49" s="1" t="str"/>
       <x:c r="V49" s="1" t="str"/>
     </x:row>
@@ -2742,7 +2838,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re30b4901b038403d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbe06ad2874344c0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2963,7 +3059,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cb4ff79b3994ca6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cb6fa0b21b74af0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3043,7 +3139,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbceece3215034054"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc74b989428e45bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3147,7 +3243,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c238f1b280d4a38"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0465cac7d6884042"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3334,7 +3430,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re52d6f4b12004848"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf01de87921354b0b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3393,7 +3489,7 @@
         <x:v>external_order_wolt_url</x:v>
       </x:c>
       <x:c r="I1" s="6" t="str">
-        <x:v>external_order_foodora_url</x:v>
+        <x:v>external_order_uber_eats_url</x:v>
       </x:c>
       <x:c r="J1" s="6" t="str">
         <x:v>phone</x:v>
@@ -3461,7 +3557,7 @@
         <x:v>https://wolt.com/fi/restaurant/spice-donor</x:v>
       </x:c>
       <x:c r="I2" s="1" t="str">
-        <x:v>https://www.foodora.fi/restaurant/spice-donor</x:v>
+        <x:v>https://www.ubereats.com/fi</x:v>
       </x:c>
       <x:c r="J2" s="1" t="str">
         <x:v>+358 9 1234 5678</x:v>
@@ -3504,7 +3600,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53888251c9184052"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reafef41827ea4aaf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update menu product image rotations
</commit_message>
<xml_diff>
--- a/outputs/menu/menu.xlsx
+++ b/outputs/menu/menu.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R1b3bc90ba0d8447d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items" sheetId="2" r:id="Reefa5ba854394f94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories" sheetId="3" r:id="Rb29171e6e1764327"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="option_groups" sheetId="4" r:id="R7f616509418d4c81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="options" sheetId="5" r:id="Ra22121c5f8bb4ec1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="specials" sheetId="6" r:id="Rc09021ada29240f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hours" sheetId="7" r:id="R4f9c26f23e704d09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="site_settings" sheetId="8" r:id="R88c8d79a1dad4ed9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R80f9e67adf0b42e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items" sheetId="2" r:id="R8e94096cad8e4ba6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories" sheetId="3" r:id="Rf08f5c044eaf450b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="option_groups" sheetId="4" r:id="R430ca64951e74300"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="options" sheetId="5" r:id="R25fc5d38e68d40b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="specials" sheetId="6" r:id="Rd7de0f8c6d464e9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hours" sheetId="7" r:id="R6a9fba453d794721"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="site_settings" sheetId="8" r:id="R51da0d332d7f4f7e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -479,12 +479,12 @@
         <x:v>Set available to TRUE/FALSE for items and visible to TRUE/FALSE for categories.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
+    <x:row r="6" ht="24" hidden="0" customHeight="1">
       <x:c r="A6" s="1" t="str">
         <x:v>Prices</x:v>
       </x:c>
       <x:c r="B6" s="7" t="str">
-        <x:v>Use numeric values in price fields. price_large is the second size. price_alt and price_alt_large support a second protein price line.</x:v>
+        <x:v>Use numeric values in price fields. price_large is the meal price (regular price + €3, including fries and Coke). price_alt and price_alt_large support a second protein price line.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -506,7 +506,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca35dd4503c84583"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0ae0d93308d47b7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -650,7 +650,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T2" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01253.jpg</x:v>
+        <x:v>assets/images/Items/Kana Döner.jpg|assets/images/Items/Kana Döner Ateria.jpg|assets/images/Items/Kana Wrap.jpg|assets/images/Items/Kana Wrap Ateria.jpg</x:v>
       </x:c>
       <x:c r="U2" s="1" t="str"/>
       <x:c r="V2" s="1" t="str"/>
@@ -698,7 +698,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T3" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01263.jpg</x:v>
+        <x:v>assets/images/Items/Halloumi–Kana Döner Ateria.jpg</x:v>
       </x:c>
       <x:c r="U3" s="1" t="str"/>
       <x:c r="V3" s="1" t="str"/>
@@ -746,7 +746,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T4" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01266.jpg</x:v>
+        <x:v>assets/images/Items/Nauta Döner.jpg|assets/images/Items/Nauta Döner Ateria.jpg</x:v>
       </x:c>
       <x:c r="U4" s="1" t="str"/>
       <x:c r="V4" s="1" t="str"/>
@@ -794,7 +794,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T5" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01283.jpg</x:v>
+        <x:v>assets/images/Items/Halloumi–Nauta Döner.jpg|assets/images/Items/Halloumi–Nauta Döner Ateria.jpg</x:v>
       </x:c>
       <x:c r="U5" s="1" t="str"/>
       <x:c r="V5" s="1" t="str"/>
@@ -842,7 +842,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T6" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01287.jpg</x:v>
+        <x:v>assets/images/Items/Kana Döner.jpg|assets/images/Items/Kana Döner Ateria.jpg|assets/images/Items/Nauta Döner.jpg|assets/images/Items/Nauta Döner Ateria.jpg</x:v>
       </x:c>
       <x:c r="U6" s="1" t="str"/>
       <x:c r="V6" s="1" t="str"/>
@@ -890,7 +890,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T7" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01291.jpg</x:v>
+        <x:v>assets/images/Items/Kasvis–Halloumi.jpg|assets/images/Items/Kasvis–Halloumi Ateria.jpg</x:v>
       </x:c>
       <x:c r="U7" s="1" t="str"/>
       <x:c r="V7" s="1" t="str"/>
@@ -938,7 +938,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T8" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01297.jpg</x:v>
+        <x:v>assets/images/Items/Vuohenjuusto &amp; Kasvis.jpg|assets/images/Items/Vuohenjuusto &amp; Kasvis Ateria.jpg</x:v>
       </x:c>
       <x:c r="U8" s="1" t="str"/>
       <x:c r="V8" s="1" t="str"/>
@@ -986,7 +986,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T9" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01301.jpg</x:v>
+        <x:v>assets/images/Items/Munakoiso–Kukkakaali Pita.jpg|assets/images/Items/Munakoiso–Kukkakaali Ateria.jpg|assets/images/Items/Munakoiso – Brokkoli Pita.jpg|assets/images/Items/Munakoiso – Brokkoli Ateria.jpg</x:v>
       </x:c>
       <x:c r="U9" s="1" t="str"/>
       <x:c r="V9" s="1" t="str"/>
@@ -1034,7 +1034,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T10" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01304.jpg</x:v>
+        <x:v>assets/images/Items/Munakoiso–Kukkakaali Pita.jpg|assets/images/Items/Munakoiso–Kukkakaali Ateria.jpg|assets/images/Items/Munakoiso – Brokkoli Pita.jpg|assets/images/Items/Munakoiso – Brokkoli Ateria.jpg</x:v>
       </x:c>
       <x:c r="U10" s="1" t="str"/>
       <x:c r="V10" s="1" t="str"/>
@@ -1082,7 +1082,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T11" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01308.jpg</x:v>
+        <x:v>assets/images/Items/Talon Vegaaninen.jpg|assets/images/Items/Talon Vegaaninen Ateria.jpg</x:v>
       </x:c>
       <x:c r="U11" s="1" t="str"/>
       <x:c r="V11" s="1" t="str"/>
@@ -1127,9 +1127,7 @@
       <x:c r="S12" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T12" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01310.jpg</x:v>
-      </x:c>
+      <x:c r="T12" s="1" t="str"/>
       <x:c r="U12" s="1" t="str"/>
       <x:c r="V12" s="1" t="str"/>
     </x:row>
@@ -1176,7 +1174,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T13" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01314.jpg</x:v>
+        <x:v>assets/images/Items/Kana Döner Mezze Bowl.jpg|assets/images/Items/Kana Döner Mezze Bowl Ateria.jpg</x:v>
       </x:c>
       <x:c r="U13" s="1" t="str"/>
       <x:c r="V13" s="1" t="str"/>
@@ -1224,7 +1222,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T14" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01318.jpg</x:v>
+        <x:v>assets/images/Items/Nauta Döner Mezze Bowl.jpg|assets/images/Items/Nauta Döner Mezze Bowl Ateria.jpg</x:v>
       </x:c>
       <x:c r="U14" s="1" t="str"/>
       <x:c r="V14" s="1" t="str"/>
@@ -1272,7 +1270,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T15" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01340.jpg</x:v>
+        <x:v>assets/images/Items/ Halloumi Mezze Bowl.jpg</x:v>
       </x:c>
       <x:c r="U15" s="1" t="str"/>
       <x:c r="V15" s="1" t="str"/>
@@ -1320,7 +1318,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T16" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01348.jpg</x:v>
+        <x:v>assets/images/Items/Vuohenjuusto Mezze Bowl.jpg|assets/images/Items/Vuohenjuusto Mezze Bowl Ateria.jpg</x:v>
       </x:c>
       <x:c r="U16" s="1" t="str"/>
       <x:c r="V16" s="1" t="str"/>
@@ -1368,7 +1366,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T17" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01353.jpg</x:v>
+        <x:v>assets/images/Items/Feta Mezze Bowl.jpg|assets/images/Items/Feta Mezze Bowl Ateria.jpg</x:v>
       </x:c>
       <x:c r="U17" s="1" t="str"/>
       <x:c r="V17" s="1" t="str"/>
@@ -1416,7 +1414,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T18" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01355.jpg</x:v>
+        <x:v>assets/images/Items/Vegan Mezze Bowl.jpg|assets/images/Items/Vegan Mezze Bowl Ateria.jpg</x:v>
       </x:c>
       <x:c r="U18" s="1" t="str"/>
       <x:c r="V18" s="1" t="str"/>
@@ -1464,7 +1462,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T19" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01360.jpg</x:v>
+        <x:v>assets/images/Items/Kana Döner Mezze Bowl.jpg|assets/images/Items/Kana Döner Mezze Bowl Ateria.jpg|assets/images/Items/Nauta Döner Mezze Bowl.jpg|assets/images/Items/Nauta Döner Mezze Bowl Ateria.jpg</x:v>
       </x:c>
       <x:c r="U19" s="1" t="str"/>
       <x:c r="V19" s="1" t="str"/>
@@ -1524,7 +1522,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T20" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01371.jpg</x:v>
+        <x:v>assets/images/Items/Kana Döner Ranskalaiset Bowl.jpg|assets/images/Items/Kana Döner Ranskalaiset Bowl Ateria.jpg|assets/images/Items/Döner Ranskalaiset Bowl Naudalla.jpg|assets/images/Items/Döner Ranskalaiset Bowl Naudalla Ateria.jpg</x:v>
       </x:c>
       <x:c r="U20" s="1" t="str"/>
       <x:c r="V20" s="1" t="str"/>
@@ -1584,7 +1582,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T21" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01374.jpg</x:v>
+        <x:v>assets/images/Items/Döner Riisi Bowl Kanalla.jpg|assets/images/Items/Döner Riisi Bowl Kanalla Ateria.jpg|assets/images/Items/Döner Riisi Bowl Naudalla.jpg|assets/images/Items/Döner Riisi Bowl Naudalla Ateria.jpg</x:v>
       </x:c>
       <x:c r="U21" s="1" t="str"/>
       <x:c r="V21" s="1" t="str"/>
@@ -1644,7 +1642,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T22" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01380.jpg</x:v>
+        <x:v>assets/images/Items/Döner Iskander Bowl Kanalla.jpg|assets/images/Items/Döner Iskander Bowl Kanalla Ateria.jpg|assets/images/Items/Döner Iskander Bowl Naudalla.jpg|assets/images/Items/Döner Iskander Bowl Naudalla Ateria.jpg</x:v>
       </x:c>
       <x:c r="U22" s="1" t="str"/>
       <x:c r="V22" s="1" t="str"/>
@@ -1691,9 +1689,7 @@
       <x:c r="S23" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T23" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01386.jpg</x:v>
-      </x:c>
+      <x:c r="T23" s="1" t="str"/>
       <x:c r="U23" s="1" t="str"/>
       <x:c r="V23" s="1" t="str"/>
     </x:row>
@@ -1737,9 +1733,7 @@
       <x:c r="S24" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T24" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01387.jpg</x:v>
-      </x:c>
+      <x:c r="T24" s="1" t="str"/>
       <x:c r="U24" s="1" t="str"/>
       <x:c r="V24" s="1" t="str"/>
     </x:row>
@@ -1783,9 +1777,7 @@
       <x:c r="S25" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T25" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01389.jpg</x:v>
-      </x:c>
+      <x:c r="T25" s="1" t="str"/>
       <x:c r="U25" s="1" t="str"/>
       <x:c r="V25" s="1" t="str"/>
     </x:row>
@@ -1830,7 +1822,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T26" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01392.jpg</x:v>
+        <x:v>assets/images/Items/Kana Döner Ranskalaiset Bowl.jpg|assets/images/Items/Kana Döner Ranskalaiset Bowl Ateria.jpg|assets/images/Items/Döner Ranskalaiset Bowl Naudalla.jpg|assets/images/Items/Döner Ranskalaiset Bowl Naudalla Ateria.jpg</x:v>
       </x:c>
       <x:c r="U26" s="1" t="str"/>
       <x:c r="V26" s="1" t="str"/>
@@ -1875,9 +1867,7 @@
       <x:c r="S27" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T27" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01394.jpg</x:v>
-      </x:c>
+      <x:c r="T27" s="1" t="str"/>
       <x:c r="U27" s="1" t="str"/>
       <x:c r="V27" s="1" t="str"/>
     </x:row>
@@ -1921,9 +1911,7 @@
       <x:c r="S28" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T28" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01395.jpg</x:v>
-      </x:c>
+      <x:c r="T28" s="1" t="str"/>
       <x:c r="U28" s="1" t="str"/>
       <x:c r="V28" s="1" t="str"/>
     </x:row>
@@ -1970,7 +1958,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T29" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01401.jpg</x:v>
+        <x:v>assets/images/Fish n Chips.png</x:v>
       </x:c>
       <x:c r="U29" s="1" t="str"/>
       <x:c r="V29" s="1" t="str"/>
@@ -2016,7 +2004,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T30" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01402.jpg</x:v>
+        <x:v>assets/images/Items/Ranskalaiset.jpg</x:v>
       </x:c>
       <x:c r="U30" s="1" t="str"/>
       <x:c r="V30" s="1" t="str"/>
@@ -2062,7 +2050,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T31" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01417.jpg</x:v>
+        <x:v>assets/images/Items/Bataattiranskalaiset.jpg</x:v>
       </x:c>
       <x:c r="U31" s="1" t="str"/>
       <x:c r="V31" s="1" t="str"/>
@@ -2108,7 +2096,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T32" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01419.jpg</x:v>
+        <x:v>assets/images/Items/Halloumiranskalaiset.jpg</x:v>
       </x:c>
       <x:c r="U32" s="1" t="str"/>
       <x:c r="V32" s="1" t="str"/>
@@ -2153,9 +2141,7 @@
       <x:c r="S33" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T33" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01423.jpg</x:v>
-      </x:c>
+      <x:c r="T33" s="1" t="str"/>
       <x:c r="U33" s="1" t="str"/>
       <x:c r="V33" s="1" t="str"/>
     </x:row>
@@ -2200,7 +2186,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T34" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01425.jpg</x:v>
+        <x:v>assets/images/Items/Falafelit &amp; Hummus.jpg</x:v>
       </x:c>
       <x:c r="U34" s="1" t="str"/>
       <x:c r="V34" s="1" t="str"/>
@@ -2246,7 +2232,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="T35" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01430.jpg</x:v>
+        <x:v>assets/images/Items/Kukkakaali &amp; Hummus .jpg|assets/images/Items/Brokkoli &amp; Hummus .jpg</x:v>
       </x:c>
       <x:c r="U35" s="1" t="str"/>
       <x:c r="V35" s="1" t="str"/>
@@ -2285,9 +2271,7 @@
       <x:c r="S36" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T36" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01433.jpg</x:v>
-      </x:c>
+      <x:c r="T36" s="1" t="str"/>
       <x:c r="U36" s="1" t="str"/>
       <x:c r="V36" s="1" t="str"/>
     </x:row>
@@ -2329,9 +2313,7 @@
       <x:c r="S37" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T37" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01438.jpg</x:v>
-      </x:c>
+      <x:c r="T37" s="1" t="str"/>
       <x:c r="U37" s="1" t="str"/>
       <x:c r="V37" s="1" t="str"/>
     </x:row>
@@ -2373,9 +2355,7 @@
       <x:c r="S38" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T38" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01447.jpg</x:v>
-      </x:c>
+      <x:c r="T38" s="1" t="str"/>
       <x:c r="U38" s="1" t="str"/>
       <x:c r="V38" s="1" t="str"/>
     </x:row>
@@ -2413,9 +2393,7 @@
       <x:c r="S39" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T39" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01456.jpg</x:v>
-      </x:c>
+      <x:c r="T39" s="1" t="str"/>
       <x:c r="U39" s="1" t="str"/>
       <x:c r="V39" s="1" t="str"/>
     </x:row>
@@ -2457,9 +2435,7 @@
       <x:c r="S40" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T40" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01462.jpg</x:v>
-      </x:c>
+      <x:c r="T40" s="1" t="str"/>
       <x:c r="U40" s="1" t="str"/>
       <x:c r="V40" s="1" t="str"/>
     </x:row>
@@ -2501,9 +2477,7 @@
       <x:c r="S41" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T41" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01466.jpg</x:v>
-      </x:c>
+      <x:c r="T41" s="1" t="str"/>
       <x:c r="U41" s="1" t="str"/>
       <x:c r="V41" s="1" t="str"/>
     </x:row>
@@ -2541,9 +2515,7 @@
       <x:c r="S42" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T42" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01468.jpg</x:v>
-      </x:c>
+      <x:c r="T42" s="1" t="str"/>
       <x:c r="U42" s="1" t="str"/>
       <x:c r="V42" s="1" t="str"/>
     </x:row>
@@ -2581,9 +2553,7 @@
       <x:c r="S43" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T43" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01469.jpg</x:v>
-      </x:c>
+      <x:c r="T43" s="1" t="str"/>
       <x:c r="U43" s="1" t="str"/>
       <x:c r="V43" s="1" t="str"/>
     </x:row>
@@ -2621,9 +2591,7 @@
       <x:c r="S44" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T44" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01473.jpg</x:v>
-      </x:c>
+      <x:c r="T44" s="1" t="str"/>
       <x:c r="U44" s="1" t="str"/>
       <x:c r="V44" s="1" t="str"/>
     </x:row>
@@ -2661,9 +2629,7 @@
       <x:c r="S45" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T45" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01481.jpg</x:v>
-      </x:c>
+      <x:c r="T45" s="1" t="str"/>
       <x:c r="U45" s="1" t="str"/>
       <x:c r="V45" s="1" t="str"/>
     </x:row>
@@ -2701,9 +2667,7 @@
       <x:c r="S46" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T46" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01488.jpg</x:v>
-      </x:c>
+      <x:c r="T46" s="1" t="str"/>
       <x:c r="U46" s="1" t="str"/>
       <x:c r="V46" s="1" t="str"/>
     </x:row>
@@ -2741,9 +2705,7 @@
       <x:c r="S47" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T47" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01492.jpg</x:v>
-      </x:c>
+      <x:c r="T47" s="1" t="str"/>
       <x:c r="U47" s="1" t="str"/>
       <x:c r="V47" s="1" t="str"/>
     </x:row>
@@ -2781,9 +2743,7 @@
       <x:c r="S48" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T48" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01501.jpg</x:v>
-      </x:c>
+      <x:c r="T48" s="1" t="str"/>
       <x:c r="U48" s="1" t="str"/>
       <x:c r="V48" s="1" t="str"/>
     </x:row>
@@ -2821,9 +2781,7 @@
       <x:c r="S49" s="9" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T49" s="1" t="str">
-        <x:v>assets/images/item-photos/TML01502.jpg</x:v>
-      </x:c>
+      <x:c r="T49" s="1" t="str"/>
       <x:c r="U49" s="1" t="str"/>
       <x:c r="V49" s="1" t="str"/>
     </x:row>
@@ -2838,7 +2796,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbe06ad2874344c0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6dfd09ff5aef481f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2879,7 +2837,7 @@
         <x:v>visible</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="15" hidden="0" customHeight="1">
+    <x:row r="2" ht="24" hidden="0" customHeight="1">
       <x:c r="A2" s="1" t="str">
         <x:v>pita_meat</x:v>
       </x:c>
@@ -2890,10 +2848,10 @@
         <x:v>Pitat &amp; wrapit - Kana &amp; naudanliha</x:v>
       </x:c>
       <x:c r="D2" s="7" t="str">
-        <x:v>Available as pita or wrap. Prices: pita / wrap.</x:v>
+        <x:v>Available as pita or wrap. Add a meal with fries and Coke for €3.</x:v>
       </x:c>
       <x:c r="E2" s="7" t="str">
-        <x:v>Saatavilla pitana tai wrappina. Hinnat: pita / wrappi.</x:v>
+        <x:v>Saatavilla pitana tai wrappina. Lisää ateria ranskalaisilla ja Coca-Colalla +3 €.</x:v>
       </x:c>
       <x:c r="F2" s="1" t="n">
         <x:v>1</x:v>
@@ -2902,7 +2860,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="15" hidden="0" customHeight="1">
+    <x:row r="3" ht="24" hidden="0" customHeight="1">
       <x:c r="A3" s="1" t="str">
         <x:v>pita_veg</x:v>
       </x:c>
@@ -2913,10 +2871,10 @@
         <x:v>Pitat &amp; wrapit - Kasvis &amp; vegaani</x:v>
       </x:c>
       <x:c r="D3" s="7" t="str">
-        <x:v>Available as pita or wrap. Prices: pita / wrap.</x:v>
+        <x:v>Available as pita or wrap. Add a meal with fries and Coke for €3.</x:v>
       </x:c>
       <x:c r="E3" s="7" t="str">
-        <x:v>Saatavilla pitana tai wrappina. Hinnat: pita / wrappi.</x:v>
+        <x:v>Saatavilla pitana tai wrappina. Lisää ateria ranskalaisilla ja Coca-Colalla +3 €.</x:v>
       </x:c>
       <x:c r="F3" s="1" t="n">
         <x:v>2</x:v>
@@ -2936,10 +2894,10 @@
         <x:v>Mezze bowlit</x:v>
       </x:c>
       <x:c r="D4" s="7" t="str">
-        <x:v>Served with fresh pide bread. Prices: regular / giant.</x:v>
+        <x:v>Served with fresh pide bread. Add a meal with fries and Coke for €3.</x:v>
       </x:c>
       <x:c r="E4" s="7" t="str">
-        <x:v>Kaikkiin annoksiin kuuluu tuoretta pide-leipää. Hinnat: normaali / jätti.</x:v>
+        <x:v>Kaikkiin annoksiin kuuluu tuoretta pide-leipää. Lisää ateria ranskalaisilla ja Coca-Colalla +3 €.</x:v>
       </x:c>
       <x:c r="F4" s="1" t="n">
         <x:v>3</x:v>
@@ -2959,10 +2917,10 @@
         <x:v>Döner bowlit</x:v>
       </x:c>
       <x:c r="D5" s="7" t="str">
-        <x:v>Prices: regular / giant.</x:v>
+        <x:v>Add a meal with fries and Coke for €3.</x:v>
       </x:c>
       <x:c r="E5" s="7" t="str">
-        <x:v>Hinnat: normaali / jätti.</x:v>
+        <x:v>Lisää ateria ranskalaisilla ja Coca-Colalla +3 €.</x:v>
       </x:c>
       <x:c r="F5" s="1" t="n">
         <x:v>4</x:v>
@@ -3059,7 +3017,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cb6fa0b21b74af0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf17212e83d804338"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3101,10 +3059,10 @@
         <x:v>size_option</x:v>
       </x:c>
       <x:c r="B2" s="1" t="str">
-        <x:v>Size</x:v>
+        <x:v>Order type</x:v>
       </x:c>
       <x:c r="C2" s="1" t="str">
-        <x:v>Koko</x:v>
+        <x:v>Tilaustapa</x:v>
       </x:c>
       <x:c r="D2" s="1" t="str">
         <x:v>single</x:v>
@@ -3139,7 +3097,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc74b989428e45bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0103f02415a849d4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3191,16 +3149,16 @@
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="1" t="str">
-        <x:v>giant</x:v>
+        <x:v>meal</x:v>
       </x:c>
       <x:c r="B3" s="1" t="str">
         <x:v>size_option</x:v>
       </x:c>
       <x:c r="C3" s="1" t="str">
-        <x:v>Giant</x:v>
+        <x:v>Meal (fries and Coke)</x:v>
       </x:c>
       <x:c r="D3" s="1" t="str">
-        <x:v>Jätti</x:v>
+        <x:v>Ateria (ranskalaiset ja Coca-Cola)</x:v>
       </x:c>
       <x:c r="E3" s="10" t="n">
         <x:v>3</x:v>
@@ -3243,7 +3201,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0465cac7d6884042"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd3b07199c104703"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3430,7 +3388,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf01de87921354b0b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raaa9db7c067d4b06"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3600,7 +3558,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reafef41827ea4aaf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R559f333b71d049ee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Expand dietary and franchise information
</commit_message>
<xml_diff>
--- a/outputs/menu/menu.xlsx
+++ b/outputs/menu/menu.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R80f9e67adf0b42e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items" sheetId="2" r:id="R8e94096cad8e4ba6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories" sheetId="3" r:id="Rf08f5c044eaf450b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="option_groups" sheetId="4" r:id="R430ca64951e74300"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="options" sheetId="5" r:id="R25fc5d38e68d40b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="specials" sheetId="6" r:id="Rd7de0f8c6d464e9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hours" sheetId="7" r:id="R6a9fba453d794721"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="site_settings" sheetId="8" r:id="R51da0d332d7f4f7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R4a329af6ca394598"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items" sheetId="2" r:id="Rec46e0b0a752424c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories" sheetId="3" r:id="Rc430dae6d68048bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="option_groups" sheetId="4" r:id="R843f98ae93de4989"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="options" sheetId="5" r:id="R8f24b9dc2ebf4d1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="specials" sheetId="6" r:id="Rf76ba627ae8a48eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hours" sheetId="7" r:id="Rcd2edf63439546a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="site_settings" sheetId="8" r:id="R7ff4a7a160c04ef5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -506,7 +506,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0ae0d93308d47b7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce1931e1ba404697"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -643,7 +643,7 @@
         <x:v>EUR</x:v>
       </x:c>
       <x:c r="Q2" s="1" t="str">
-        <x:v>L,(G)</x:v>
+        <x:v>L,(G),H</x:v>
       </x:c>
       <x:c r="R2" s="1" t="str"/>
       <x:c r="S2" s="9" t="b">
@@ -691,7 +691,7 @@
         <x:v>EUR</x:v>
       </x:c>
       <x:c r="Q3" s="1" t="str">
-        <x:v>L,(G)</x:v>
+        <x:v>L,(G),H</x:v>
       </x:c>
       <x:c r="R3" s="1" t="str"/>
       <x:c r="S3" s="9" t="b">
@@ -739,7 +739,7 @@
         <x:v>EUR</x:v>
       </x:c>
       <x:c r="Q4" s="1" t="str">
-        <x:v>L,(G)</x:v>
+        <x:v>L,(G),H</x:v>
       </x:c>
       <x:c r="R4" s="1" t="str"/>
       <x:c r="S4" s="9" t="b">
@@ -787,7 +787,7 @@
         <x:v>EUR</x:v>
       </x:c>
       <x:c r="Q5" s="1" t="str">
-        <x:v>L,(G)</x:v>
+        <x:v>L,(G),H</x:v>
       </x:c>
       <x:c r="R5" s="1" t="str"/>
       <x:c r="S5" s="9" t="b">
@@ -835,7 +835,7 @@
         <x:v>EUR</x:v>
       </x:c>
       <x:c r="Q6" s="1" t="str">
-        <x:v>L,(G)</x:v>
+        <x:v>L,(G),H</x:v>
       </x:c>
       <x:c r="R6" s="1" t="str"/>
       <x:c r="S6" s="9" t="b">
@@ -1122,7 +1122,9 @@
       <x:c r="P12" s="1" t="str">
         <x:v>EUR</x:v>
       </x:c>
-      <x:c r="Q12" s="1" t="str"/>
+      <x:c r="Q12" s="1" t="str">
+        <x:v>H</x:v>
+      </x:c>
       <x:c r="R12" s="1" t="str"/>
       <x:c r="S12" s="9" t="b">
         <x:v>1</x:v>
@@ -1167,7 +1169,7 @@
         <x:v>EUR</x:v>
       </x:c>
       <x:c r="Q13" s="1" t="str">
-        <x:v>L,(G)</x:v>
+        <x:v>L,(G),H</x:v>
       </x:c>
       <x:c r="R13" s="1" t="str"/>
       <x:c r="S13" s="9" t="b">
@@ -1215,7 +1217,7 @@
         <x:v>EUR</x:v>
       </x:c>
       <x:c r="Q14" s="1" t="str">
-        <x:v>L,(G)</x:v>
+        <x:v>L,(G),H</x:v>
       </x:c>
       <x:c r="R14" s="1" t="str"/>
       <x:c r="S14" s="9" t="b">
@@ -1455,7 +1457,7 @@
         <x:v>EUR</x:v>
       </x:c>
       <x:c r="Q19" s="1" t="str">
-        <x:v>L,(G)</x:v>
+        <x:v>L,(G),H</x:v>
       </x:c>
       <x:c r="R19" s="1" t="str"/>
       <x:c r="S19" s="9" t="b">
@@ -1515,7 +1517,7 @@
         <x:v>EUR</x:v>
       </x:c>
       <x:c r="Q20" s="1" t="str">
-        <x:v>L,(G)</x:v>
+        <x:v>L,(G),H</x:v>
       </x:c>
       <x:c r="R20" s="1" t="str"/>
       <x:c r="S20" s="9" t="b">
@@ -1575,7 +1577,7 @@
         <x:v>EUR</x:v>
       </x:c>
       <x:c r="Q21" s="1" t="str">
-        <x:v>L,(G)</x:v>
+        <x:v>L,(G),H</x:v>
       </x:c>
       <x:c r="R21" s="1" t="str"/>
       <x:c r="S21" s="9" t="b">
@@ -1635,7 +1637,7 @@
         <x:v>EUR</x:v>
       </x:c>
       <x:c r="Q22" s="1" t="str">
-        <x:v>L,(G)</x:v>
+        <x:v>L,(G),H</x:v>
       </x:c>
       <x:c r="R22" s="1" t="str"/>
       <x:c r="S22" s="9" t="b">
@@ -1728,7 +1730,9 @@
       <x:c r="P24" s="1" t="str">
         <x:v>EUR</x:v>
       </x:c>
-      <x:c r="Q24" s="1" t="str"/>
+      <x:c r="Q24" s="1" t="str">
+        <x:v>H</x:v>
+      </x:c>
       <x:c r="R24" s="1" t="str"/>
       <x:c r="S24" s="9" t="b">
         <x:v>1</x:v>
@@ -1772,7 +1776,9 @@
       <x:c r="P25" s="1" t="str">
         <x:v>EUR</x:v>
       </x:c>
-      <x:c r="Q25" s="1" t="str"/>
+      <x:c r="Q25" s="1" t="str">
+        <x:v>H</x:v>
+      </x:c>
       <x:c r="R25" s="1" t="str"/>
       <x:c r="S25" s="9" t="b">
         <x:v>1</x:v>
@@ -1815,7 +1821,7 @@
         <x:v>EUR</x:v>
       </x:c>
       <x:c r="Q26" s="1" t="str">
-        <x:v>L,G</x:v>
+        <x:v>L,G,H</x:v>
       </x:c>
       <x:c r="R26" s="1" t="str"/>
       <x:c r="S26" s="9" t="b">
@@ -1906,7 +1912,9 @@
       <x:c r="P28" s="1" t="str">
         <x:v>EUR</x:v>
       </x:c>
-      <x:c r="Q28" s="1" t="str"/>
+      <x:c r="Q28" s="1" t="str">
+        <x:v>H</x:v>
+      </x:c>
       <x:c r="R28" s="1" t="str"/>
       <x:c r="S28" s="9" t="b">
         <x:v>1</x:v>
@@ -2796,7 +2804,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6dfd09ff5aef481f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7eb6661e4bbb483b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2848,10 +2856,10 @@
         <x:v>Pitat &amp; wrapit - Kana &amp; naudanliha</x:v>
       </x:c>
       <x:c r="D2" s="7" t="str">
-        <x:v>Available as pita or wrap. Add a meal with fries and Coke for €3.</x:v>
+        <x:v>Every item in this section can be served as either a pita or a wrap. Add a meal with fries and Coke for €3.</x:v>
       </x:c>
       <x:c r="E2" s="7" t="str">
-        <x:v>Saatavilla pitana tai wrappina. Lisää ateria ranskalaisilla ja Coca-Colalla +3 €.</x:v>
+        <x:v>Jokainen tämän osion annos voidaan tarjoilla joko pitana tai wrappina. Lisää ateria ranskalaisilla ja Coca-Colalla +3 €.</x:v>
       </x:c>
       <x:c r="F2" s="1" t="n">
         <x:v>1</x:v>
@@ -2871,10 +2879,10 @@
         <x:v>Pitat &amp; wrapit - Kasvis &amp; vegaani</x:v>
       </x:c>
       <x:c r="D3" s="7" t="str">
-        <x:v>Available as pita or wrap. Add a meal with fries and Coke for €3.</x:v>
+        <x:v>Every item in this section can be served as either a pita or a wrap. Add a meal with fries and Coke for €3.</x:v>
       </x:c>
       <x:c r="E3" s="7" t="str">
-        <x:v>Saatavilla pitana tai wrappina. Lisää ateria ranskalaisilla ja Coca-Colalla +3 €.</x:v>
+        <x:v>Jokainen tämän osion annos voidaan tarjoilla joko pitana tai wrappina. Lisää ateria ranskalaisilla ja Coca-Colalla +3 €.</x:v>
       </x:c>
       <x:c r="F3" s="1" t="n">
         <x:v>2</x:v>
@@ -3017,7 +3025,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf17212e83d804338"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R493983bdebe24417"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3097,7 +3105,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0103f02415a849d4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2eaf62b277c042b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3201,7 +3209,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd3b07199c104703"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb5ac37e2a2a4e09"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3388,7 +3396,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raaa9db7c067d4b06"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e8ccd0d5b514092"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3558,7 +3566,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R559f333b71d049ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26c053397ae845fc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Prepare Spice Donor for Cloudflare launch
</commit_message>
<xml_diff>
--- a/outputs/menu/menu.xlsx
+++ b/outputs/menu/menu.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R4a329af6ca394598"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items" sheetId="2" r:id="Rec46e0b0a752424c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories" sheetId="3" r:id="Rc430dae6d68048bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="option_groups" sheetId="4" r:id="R843f98ae93de4989"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="options" sheetId="5" r:id="R8f24b9dc2ebf4d1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="specials" sheetId="6" r:id="Rf76ba627ae8a48eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hours" sheetId="7" r:id="Rcd2edf63439546a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="site_settings" sheetId="8" r:id="R7ff4a7a160c04ef5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R09150d3ed7e049f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items" sheetId="2" r:id="Rdc09b83e6aeb439a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories" sheetId="3" r:id="R08226921d4824179"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="option_groups" sheetId="4" r:id="Rd3137d5f5c364e8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="options" sheetId="5" r:id="R28dc1d1978c740a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="specials" sheetId="6" r:id="Ra8fab4c7307d4ac6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hours" sheetId="7" r:id="Rb0cf7503ef54493e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="site_settings" sheetId="8" r:id="Rcf0e91b949d24b81"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -506,7 +506,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce1931e1ba404697"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77af4c450e504669"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2804,7 +2804,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7eb6661e4bbb483b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70cbc6bbb53249a7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3025,7 +3025,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R493983bdebe24417"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9df22786df54fd5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3105,7 +3105,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2eaf62b277c042b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43947aa750a94cd6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3209,7 +3209,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb5ac37e2a2a4e09"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63707299cd3c4fde"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3396,7 +3396,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e8ccd0d5b514092"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bfd040e0b564778"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3522,27 +3522,25 @@
       <x:c r="H2" s="1" t="str">
         <x:v>https://wolt.com/fi/restaurant/spice-donor</x:v>
       </x:c>
-      <x:c r="I2" s="1" t="str">
-        <x:v>https://www.ubereats.com/fi</x:v>
-      </x:c>
-      <x:c r="J2" s="1" t="str">
-        <x:v>+358 9 1234 5678</x:v>
-      </x:c>
+      <x:c r="I2" s="1" t="str"/>
+      <x:c r="J2" s="1" t="str"/>
       <x:c r="K2" s="1" t="str">
         <x:v>info@spicedonor.fi</x:v>
       </x:c>
       <x:c r="L2" s="1" t="str">
-        <x:v>Malminkaari 9</x:v>
-      </x:c>
-      <x:c r="M2" s="1" t="str"/>
+        <x:v>Kauppakeskus Forum (food court)</x:v>
+      </x:c>
+      <x:c r="M2" s="1" t="str">
+        <x:v>Mannerheimintie 20</x:v>
+      </x:c>
       <x:c r="N2" s="1" t="str">
         <x:v>Helsinki</x:v>
       </x:c>
       <x:c r="O2" s="1" t="str">
-        <x:v>00700</x:v>
+        <x:v>00100</x:v>
       </x:c>
       <x:c r="P2" s="1" t="str">
-        <x:v>https://maps.google.com/maps?q=Malminkaari+9,+00700+Helsinki&amp;output=embed</x:v>
+        <x:v>https://maps.google.com/maps?q=Kauppakeskus+Forum,+Mannerheimintie+20,+00100+Helsinki&amp;output=embed</x:v>
       </x:c>
       <x:c r="Q2" s="1" t="str">
         <x:v>https://instagram.com/spicedonor</x:v>
@@ -3566,7 +3564,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26c053397ae845fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R690778a40ac94f75"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>